<commit_message>
Modification of list files dates
</commit_message>
<xml_diff>
--- a/scripts/list_dates_files.xlsx
+++ b/scripts/list_dates_files.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Backup_Tomy\Data\Kivu_monitoring\Government\lake-kivu-ctd-profiles\scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Backup_Tomy\Data\Kivu_monitoring\CTD\lake-kivu-ctd-profiles\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">list_dates_files!$A$1:$C$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -7125,7 +7125,7 @@
   <dimension ref="A1:C2093"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.21875" customWidth="1"/>
+    <col min="2" max="2" width="48.109375" customWidth="1"/>
     <col min="3" max="3" width="29.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -27458,46 +27458,46 @@
       </c>
     </row>
     <row r="1849" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1849">
+      <c r="A1849" s="2">
         <v>531</v>
       </c>
-      <c r="B1849" t="s">
+      <c r="B1849" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="C1849" s="1">
+      <c r="C1849" s="3">
         <v>43741.447557870371</v>
       </c>
     </row>
     <row r="1850" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1850">
+      <c r="A1850" s="2">
         <v>537</v>
       </c>
-      <c r="B1850" t="s">
+      <c r="B1850" s="2" t="s">
         <v>540</v>
       </c>
-      <c r="C1850" s="1">
+      <c r="C1850" s="3">
         <v>43766.376875000002</v>
       </c>
     </row>
     <row r="1851" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1851">
+      <c r="A1851" s="2">
         <v>538</v>
       </c>
-      <c r="B1851" t="s">
+      <c r="B1851" s="2" t="s">
         <v>541</v>
       </c>
-      <c r="C1851" s="1">
+      <c r="C1851" s="3">
         <v>43766.457986111112</v>
       </c>
     </row>
     <row r="1852" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1852">
+      <c r="A1852" s="2">
         <v>539</v>
       </c>
-      <c r="B1852" t="s">
+      <c r="B1852" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="C1852" s="1">
+      <c r="C1852" s="3">
         <v>43766.549537037034</v>
       </c>
     </row>
@@ -28030,35 +28030,35 @@
       </c>
     </row>
     <row r="1901" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1901">
+      <c r="A1901" s="2">
         <v>643</v>
       </c>
-      <c r="B1901" t="s">
+      <c r="B1901" s="2" t="s">
         <v>646</v>
       </c>
-      <c r="C1901" s="1">
+      <c r="C1901" s="3">
         <v>44261.377141203702</v>
       </c>
     </row>
     <row r="1902" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1902">
+      <c r="A1902" s="2">
         <v>644</v>
       </c>
-      <c r="B1902" t="s">
+      <c r="B1902" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="C1902" s="1">
+      <c r="C1902" s="3">
         <v>44261.417500000003</v>
       </c>
     </row>
     <row r="1903" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1903">
+      <c r="A1903" s="2">
         <v>645</v>
       </c>
-      <c r="B1903" t="s">
+      <c r="B1903" s="2" t="s">
         <v>648</v>
       </c>
-      <c r="C1903" s="1">
+      <c r="C1903" s="3">
         <v>44261.452662037038</v>
       </c>
     </row>

</xml_diff>